<commit_message>
deploy: main → 01f7545256c4330650e0b534102108500805f0b6
</commit_message>
<xml_diff>
--- a/StructureDefinition-tk-administrator-role.xlsx
+++ b/StructureDefinition-tk-administrator-role.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$28</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="290">
   <si>
     <t>Property</t>
   </si>
@@ -540,7 +540,7 @@
 </t>
   </si>
   <si>
-    <t>Whether this practitioner role record is in active use</t>
+    <t>Om behörigheten gäller (false = återkallad)</t>
   </si>
   <si>
     <t xml:space="preserve"> Whether this practitioner role record is in active use. Some systems may use this property to mark non-active practitioners, such as those that are not currently employed.</t>
@@ -553,6 +553,9 @@
   </si>
   <si>
     <t>This resource is generally assumed to be active if no value is provided for the active element</t>
+  </si>
+  <si>
+    <t>REQ-ADM-4</t>
   </si>
   <si>
     <t>FiveWs.status</t>
@@ -574,7 +577,7 @@
 </t>
   </si>
   <si>
-    <t>The period during which the practitioner is authorized to perform in these role(s)</t>
+    <t>Behörighetens giltighetsperiod</t>
   </si>
   <si>
     <t>The period during which the person is authorized to act as a practitioner in these role(s) for the organization.</t>
@@ -596,6 +599,97 @@
   </si>
   <si>
     <t>(ServD maps Practitioners and Organizations via another entity, so this concept is not available)</t>
+  </si>
+  <si>
+    <t>PractitionerRole.period.id</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1
+</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>PractitionerRole.period.extension</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and managable, there is a strict set of governance applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>PractitionerRole.period.start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dateTime
+</t>
+  </si>
+  <si>
+    <t>Starting time with inclusive boundary</t>
+  </si>
+  <si>
+    <t>The start of the period. The boundary is inclusive.</t>
+  </si>
+  <si>
+    <t>If the low element is missing, the meaning is that the low boundary is not known.</t>
+  </si>
+  <si>
+    <t>Period.start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per-1
+</t>
+  </si>
+  <si>
+    <t>DR.1</t>
+  </si>
+  <si>
+    <t>./low</t>
+  </si>
+  <si>
+    <t>PractitionerRole.period.end</t>
+  </si>
+  <si>
+    <t>End time with inclusive boundary, if not ongoing</t>
+  </si>
+  <si>
+    <t>The end of the period. If the end of the period is missing, it means no end was known or planned at the time the instance was created. The start may be in the past, and the end date in the future, which means that period is expected/planned to end at that time.</t>
+  </si>
+  <si>
+    <t>The end value includes any matching date/time. i.e. 2012-02-03T10:00:00 is in a period that has an end value of 2012-02-03.</t>
+  </si>
+  <si>
+    <t>If the end of the period is missing, it means that the period is ongoing</t>
+  </si>
+  <si>
+    <t>Period.end</t>
+  </si>
+  <si>
+    <t>DR.2</t>
+  </si>
+  <si>
+    <t>./high</t>
   </si>
   <si>
     <t>PractitionerRole.practitioner</t>
@@ -835,9 +929,6 @@
   <si>
     <t>Organizations have multiple systems that provide various services and may also be different for practitioners too.
 So the endpoint satisfies the need to be able to define the technical connection details for how to connect to them, and for what purpose.</t>
-  </si>
-  <si>
-    <t>n/a</t>
   </si>
 </sst>
 </file>
@@ -1162,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP24"/>
+  <dimension ref="A1:AP28"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="28.1953125" customWidth="true" bestFit="true"/>
@@ -1193,7 +1284,7 @@
     <col min="26" max="26" width="54.09375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="29.0546875" customWidth="true" bestFit="true" hidden="true"/>
@@ -2536,7 +2627,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="12" hidden="true">
+    <row r="12">
       <c r="A12" t="s" s="2">
         <v>164</v>
       </c>
@@ -2555,7 +2646,7 @@
         <v>93</v>
       </c>
       <c r="H12" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I12" t="s" s="2">
         <v>80</v>
@@ -2642,30 +2733,30 @@
         <v>106</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>80</v>
+        <v>171</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AM12" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AN12" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AO12" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AP12" t="s" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="13" hidden="true">
+    <row r="13">
       <c r="A13" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2679,7 +2770,7 @@
         <v>93</v>
       </c>
       <c r="H13" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I13" t="s" s="2">
         <v>80</v>
@@ -2688,19 +2779,19 @@
         <v>94</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="O13" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P13" t="s" s="2">
         <v>80</v>
@@ -2749,7 +2840,7 @@
         <v>80</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>81</v>
@@ -2764,30 +2855,30 @@
         <v>106</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>80</v>
+        <v>171</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AM13" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AO13" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP13" t="s" s="2">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="14">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2801,16 +2892,16 @@
         <v>93</v>
       </c>
       <c r="H14" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I14" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>186</v>
+        <v>95</v>
       </c>
       <c r="L14" t="s" s="2">
         <v>187</v>
@@ -2867,7 +2958,7 @@
         <v>80</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>81</v>
@@ -2876,13 +2967,13 @@
         <v>93</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>80</v>
+        <v>190</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>189</v>
+        <v>80</v>
       </c>
       <c r="AL14" t="s" s="2">
         <v>80</v>
@@ -2891,7 +2982,7 @@
         <v>80</v>
       </c>
       <c r="AN14" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AO14" t="s" s="2">
         <v>80</v>
@@ -2900,43 +2991,45 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="H15" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="I15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>192</v>
+        <v>142</v>
       </c>
       <c r="L15" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="M15" t="s" s="2">
         <v>193</v>
       </c>
-      <c r="M15" t="s" s="2">
-        <v>194</v>
-      </c>
-      <c r="N15" s="2"/>
+      <c r="N15" t="s" s="2">
+        <v>145</v>
+      </c>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>80</v>
@@ -2973,43 +3066,43 @@
         <v>80</v>
       </c>
       <c r="AB15" t="s" s="2">
-        <v>80</v>
+        <v>194</v>
       </c>
       <c r="AC15" t="s" s="2">
-        <v>80</v>
+        <v>195</v>
       </c>
       <c r="AD15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE15" t="s" s="2">
-        <v>80</v>
+        <v>196</v>
       </c>
       <c r="AF15" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="AG15" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="AK15" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM15" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN15" t="s" s="2">
         <v>191</v>
-      </c>
-      <c r="AG15" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH15" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI15" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ15" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="AK15" t="s" s="2">
-        <v>195</v>
-      </c>
-      <c r="AL15" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AN15" t="s" s="2">
-        <v>196</v>
       </c>
       <c r="AO15" t="s" s="2">
         <v>80</v>
@@ -3020,10 +3113,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3031,7 +3124,7 @@
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s" s="2">
         <v>93</v>
@@ -3046,20 +3139,18 @@
         <v>94</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>201</v>
-      </c>
-      <c r="O16" t="s" s="2">
         <v>202</v>
       </c>
+      <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
         <v>80</v>
       </c>
@@ -3083,44 +3174,46 @@
         <v>80</v>
       </c>
       <c r="X16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF16" t="s" s="2">
         <v>203</v>
       </c>
-      <c r="Y16" s="2"/>
-      <c r="Z16" t="s" s="2">
+      <c r="AG16" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AI16" t="s" s="2">
         <v>204</v>
-      </c>
-      <c r="AA16" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB16" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC16" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD16" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE16" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF16" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="AG16" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH16" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI16" t="s" s="2">
-        <v>80</v>
       </c>
       <c r="AJ16" t="s" s="2">
         <v>106</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="AL16" t="s" s="2">
         <v>80</v>
@@ -3132,18 +3225,18 @@
         <v>206</v>
       </c>
       <c r="AO16" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP16" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="2">
         <v>207</v>
       </c>
-      <c r="AP16" t="s" s="2">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="17" hidden="true">
-      <c r="A17" t="s" s="2">
-        <v>208</v>
-      </c>
       <c r="B17" t="s" s="2">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3154,10 +3247,10 @@
         <v>81</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I17" t="s" s="2">
         <v>80</v>
@@ -3166,22 +3259,24 @@
         <v>94</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L17" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="M17" t="s" s="2">
         <v>209</v>
       </c>
-      <c r="M17" t="s" s="2">
+      <c r="N17" t="s" s="2">
         <v>210</v>
-      </c>
-      <c r="N17" t="s" s="2">
-        <v>211</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q17" s="2"/>
+      <c r="Q17" t="s" s="2">
+        <v>211</v>
+      </c>
       <c r="R17" t="s" s="2">
         <v>80</v>
       </c>
@@ -3201,40 +3296,40 @@
         <v>80</v>
       </c>
       <c r="X17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="Y17" t="s" s="2">
-        <v>213</v>
-      </c>
-      <c r="Z17" t="s" s="2">
-        <v>214</v>
-      </c>
-      <c r="AA17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>208</v>
-      </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI17" t="s" s="2">
-        <v>80</v>
+        <v>204</v>
       </c>
       <c r="AJ17" t="s" s="2">
         <v>106</v>
@@ -3246,24 +3341,24 @@
         <v>80</v>
       </c>
       <c r="AM17" t="s" s="2">
+        <v>213</v>
+      </c>
+      <c r="AN17" t="s" s="2">
+        <v>214</v>
+      </c>
+      <c r="AO17" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP17" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="2">
         <v>215</v>
       </c>
-      <c r="AN17" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="AO17" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP17" t="s" s="2">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="18" hidden="true">
-      <c r="A18" t="s" s="2">
-        <v>218</v>
-      </c>
       <c r="B18" t="s" s="2">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3274,10 +3369,10 @@
         <v>81</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H18" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I18" t="s" s="2">
         <v>80</v>
@@ -3286,13 +3381,13 @@
         <v>94</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3343,13 +3438,13 @@
         <v>80</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI18" t="s" s="2">
         <v>80</v>
@@ -3358,30 +3453,30 @@
         <v>106</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>80</v>
+        <v>219</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>222</v>
+        <v>80</v>
       </c>
       <c r="AM18" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="AO18" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP18" t="s" s="2">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="19" hidden="true">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" t="s" s="2">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3392,25 +3487,25 @@
         <v>81</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H19" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3461,13 +3556,13 @@
         <v>80</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="AI19" t="s" s="2">
         <v>80</v>
@@ -3476,16 +3571,16 @@
         <v>106</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>80</v>
+        <v>225</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>229</v>
+        <v>80</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="AO19" t="s" s="2">
         <v>80</v>
@@ -3494,12 +3589,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" hidden="true">
+    <row r="20">
       <c r="A20" t="s" s="2">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3507,32 +3602,34 @@
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="L20" t="s" s="2">
+        <v>229</v>
+      </c>
+      <c r="M20" t="s" s="2">
+        <v>230</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="O20" t="s" s="2">
         <v>232</v>
-      </c>
-      <c r="L20" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="N20" s="2"/>
-      <c r="O20" t="s" s="2">
-        <v>235</v>
       </c>
       <c r="P20" t="s" s="2">
         <v>80</v>
@@ -3557,13 +3654,11 @@
         <v>80</v>
       </c>
       <c r="X20" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y20" t="s" s="2">
-        <v>80</v>
-      </c>
+        <v>233</v>
+      </c>
+      <c r="Y20" s="2"/>
       <c r="Z20" t="s" s="2">
-        <v>80</v>
+        <v>234</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>80</v>
@@ -3581,7 +3676,7 @@
         <v>80</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
@@ -3596,30 +3691,30 @@
         <v>106</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="AL20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>80</v>
+        <v>235</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>80</v>
+        <v>236</v>
       </c>
       <c r="AO20" t="s" s="2">
-        <v>80</v>
+        <v>237</v>
       </c>
       <c r="AP20" t="s" s="2">
-        <v>80</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3639,19 +3734,19 @@
         <v>80</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>198</v>
+        <v>228</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -3677,13 +3772,13 @@
         <v>80</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>203</v>
+        <v>242</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>80</v>
@@ -3701,7 +3796,7 @@
         <v>80</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
@@ -3722,24 +3817,24 @@
         <v>80</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>80</v>
+        <v>245</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="AO21" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP21" t="s" s="2">
-        <v>80</v>
+        <v>247</v>
       </c>
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3759,23 +3854,19 @@
         <v>80</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>198</v>
+        <v>249</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>245</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>246</v>
-      </c>
-      <c r="O22" t="s" s="2">
-        <v>247</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>80</v>
       </c>
@@ -3799,13 +3890,13 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>80</v>
@@ -3823,7 +3914,7 @@
         <v>80</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -3841,27 +3932,27 @@
         <v>80</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>80</v>
+        <v>252</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP22" t="s" s="2">
-        <v>80</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3884,17 +3975,15 @@
         <v>80</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>252</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>253</v>
-      </c>
+        <v>258</v>
+      </c>
+      <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>80</v>
@@ -3943,7 +4032,7 @@
         <v>80</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>81</v>
@@ -3964,10 +4053,10 @@
         <v>80</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>80</v>
+        <v>259</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="AO23" t="s" s="2">
         <v>80</v>
@@ -3978,10 +4067,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4004,17 +4093,17 @@
         <v>80</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" t="s" s="2">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>80</v>
@@ -4063,7 +4152,7 @@
         <v>80</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>81</v>
@@ -4087,7 +4176,7 @@
         <v>80</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>260</v>
+        <v>80</v>
       </c>
       <c r="AO24" t="s" s="2">
         <v>80</v>
@@ -4096,8 +4185,490 @@
         <v>80</v>
       </c>
     </row>
+    <row r="25" hidden="true">
+      <c r="A25" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="B25" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K25" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="L25" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="M25" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="O25" s="2"/>
+      <c r="P25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q25" s="2"/>
+      <c r="R25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X25" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="Y25" t="s" s="2">
+        <v>270</v>
+      </c>
+      <c r="Z25" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="AA25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF25" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="AG25" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH25" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ25" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AK25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN25" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="AO25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP25" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" hidden="true">
+      <c r="A26" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="B26" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K26" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="L26" t="s" s="2">
+        <v>274</v>
+      </c>
+      <c r="M26" t="s" s="2">
+        <v>275</v>
+      </c>
+      <c r="N26" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="O26" t="s" s="2">
+        <v>277</v>
+      </c>
+      <c r="P26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q26" s="2"/>
+      <c r="R26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X26" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="Y26" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="Z26" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AA26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF26" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="AG26" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH26" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ26" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AK26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN26" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="AO26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP26" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" hidden="true">
+      <c r="A27" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="B27" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K27" t="s" s="2">
+        <v>280</v>
+      </c>
+      <c r="L27" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="M27" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="O27" s="2"/>
+      <c r="P27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q27" s="2"/>
+      <c r="R27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF27" t="s" s="2">
+        <v>279</v>
+      </c>
+      <c r="AG27" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ27" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AK27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN27" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="AO27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP27" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" hidden="true">
+      <c r="A28" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="B28" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G28" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K28" t="s" s="2">
+        <v>286</v>
+      </c>
+      <c r="L28" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="M28" t="s" s="2">
+        <v>288</v>
+      </c>
+      <c r="N28" s="2"/>
+      <c r="O28" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="P28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q28" s="2"/>
+      <c r="R28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF28" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="AK28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN28" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="AO28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP28" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AP24">
+  <autoFilter ref="A1:AP28">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -4107,7 +4678,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI23">
+  <conditionalFormatting sqref="A2:AI27">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>